<commit_message>
EGO Master LIVE: Excel basics with dropdowns
</commit_message>
<xml_diff>
--- a/ego/EGO-Inventory-Upload-Template.xlsx
+++ b/ego/EGO-Inventory-Upload-Template.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>EGO-INV-2</t>
+          <t>EGO-INV-3</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>1 Categories, 2 Collections (with the box size), 3 Warehouses, 4 Designs &amp; stock. Each sheet uses names from the sheet before it, written exactly the same.</t>
+          <t>1 Categories, 2 Collections (with the box size), 3 Warehouses, 4 Designs &amp; stock. Each sheet picks names from the sheets before it with a dropdown, so fill them in that order.</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB60"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -992,35 +992,15 @@
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="19" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="17" customWidth="1" min="22" max="22"/>
-    <col width="16" customWidth="1" min="23" max="23"/>
-    <col width="16" customWidth="1" min="24" max="24"/>
-    <col width="31" customWidth="1" min="25" max="25"/>
-    <col width="30" customWidth="1" min="26" max="26"/>
-    <col width="16" customWidth="1" min="27" max="27"/>
-    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Category (as on the Categories sheet) *</t>
+          <t>Category (pick from the Categories sheet) *</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
@@ -1045,117 +1025,17 @@
       </c>
       <c r="F1" s="8" t="inlineStr">
         <is>
-          <t>Weight per box (kg)</t>
+          <t>Size (mm)</t>
         </is>
       </c>
       <c r="G1" s="8" t="inlineStr">
         <is>
-          <t>Boxes per pallet</t>
+          <t>Thickness</t>
         </is>
       </c>
       <c r="H1" s="8" t="inlineStr">
         <is>
-          <t>Price per sq ft (₹)</t>
-        </is>
-      </c>
-      <c r="I1" s="8" t="inlineStr">
-        <is>
-          <t>Size (mm)</t>
-        </is>
-      </c>
-      <c r="J1" s="8" t="inlineStr">
-        <is>
-          <t>Thickness</t>
-        </is>
-      </c>
-      <c r="K1" s="8" t="inlineStr">
-        <is>
           <t>Wear layer</t>
-        </is>
-      </c>
-      <c r="L1" s="8" t="inlineStr">
-        <is>
-          <t>Construction or layers</t>
-        </is>
-      </c>
-      <c r="M1" s="8" t="inlineStr">
-        <is>
-          <t>Core or base</t>
-        </is>
-      </c>
-      <c r="N1" s="8" t="inlineStr">
-        <is>
-          <t>AC rating</t>
-        </is>
-      </c>
-      <c r="O1" s="8" t="inlineStr">
-        <is>
-          <t>Class of use</t>
-        </is>
-      </c>
-      <c r="P1" s="8" t="inlineStr">
-        <is>
-          <t>Surface or finish</t>
-        </is>
-      </c>
-      <c r="Q1" s="8" t="inlineStr">
-        <is>
-          <t>Edges</t>
-        </is>
-      </c>
-      <c r="R1" s="8" t="inlineStr">
-        <is>
-          <t>Click system</t>
-        </is>
-      </c>
-      <c r="S1" s="8" t="inlineStr">
-        <is>
-          <t>Underlay</t>
-        </is>
-      </c>
-      <c r="T1" s="8" t="inlineStr">
-        <is>
-          <t>Water resistance</t>
-        </is>
-      </c>
-      <c r="U1" s="8" t="inlineStr">
-        <is>
-          <t>Fire rating</t>
-        </is>
-      </c>
-      <c r="V1" s="8" t="inlineStr">
-        <is>
-          <t>Slip resistance</t>
-        </is>
-      </c>
-      <c r="W1" s="8" t="inlineStr">
-        <is>
-          <t>Acoustics</t>
-        </is>
-      </c>
-      <c r="X1" s="8" t="inlineStr">
-        <is>
-          <t>Emissions</t>
-        </is>
-      </c>
-      <c r="Y1" s="8" t="inlineStr">
-        <is>
-          <t>Warranty, residential (years)</t>
-        </is>
-      </c>
-      <c r="Z1" s="8" t="inlineStr">
-        <is>
-          <t>Warranty, commercial (years)</t>
-        </is>
-      </c>
-      <c r="AA1" s="8" t="inlineStr">
-        <is>
-          <t>Catalogue link</t>
-        </is>
-      </c>
-      <c r="AB1" s="8" t="inlineStr">
-        <is>
-          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -1177,45 +1057,21 @@
       <c r="E2" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="F2" s="6" t="inlineStr"/>
-      <c r="G2" s="6" t="inlineStr"/>
-      <c r="H2" s="6" t="inlineStr"/>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>1219 x 178</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>2.0mm</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>0.1mm</t>
         </is>
       </c>
-      <c r="L2" s="6" t="inlineStr"/>
-      <c r="M2" s="6" t="inlineStr"/>
-      <c r="N2" s="6" t="inlineStr"/>
-      <c r="O2" s="6" t="inlineStr"/>
-      <c r="P2" s="6" t="inlineStr"/>
-      <c r="Q2" s="6" t="inlineStr"/>
-      <c r="R2" s="6" t="inlineStr"/>
-      <c r="S2" s="6" t="inlineStr"/>
-      <c r="T2" s="6" t="inlineStr"/>
-      <c r="U2" s="6" t="inlineStr"/>
-      <c r="V2" s="6" t="inlineStr"/>
-      <c r="W2" s="6" t="inlineStr"/>
-      <c r="X2" s="6" t="inlineStr"/>
-      <c r="Y2" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="Z2" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA2" s="6" t="inlineStr"/>
-      <c r="AB2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n"/>
@@ -1226,26 +1082,6 @@
       <c r="F3" s="7" t="n"/>
       <c r="G3" s="7" t="n"/>
       <c r="H3" s="7" t="n"/>
-      <c r="I3" s="7" t="n"/>
-      <c r="J3" s="7" t="n"/>
-      <c r="K3" s="7" t="n"/>
-      <c r="L3" s="7" t="n"/>
-      <c r="M3" s="7" t="n"/>
-      <c r="N3" s="7" t="n"/>
-      <c r="O3" s="7" t="n"/>
-      <c r="P3" s="7" t="n"/>
-      <c r="Q3" s="7" t="n"/>
-      <c r="R3" s="7" t="n"/>
-      <c r="S3" s="7" t="n"/>
-      <c r="T3" s="7" t="n"/>
-      <c r="U3" s="7" t="n"/>
-      <c r="V3" s="7" t="n"/>
-      <c r="W3" s="7" t="n"/>
-      <c r="X3" s="7" t="n"/>
-      <c r="Y3" s="7" t="n"/>
-      <c r="Z3" s="7" t="n"/>
-      <c r="AA3" s="7" t="n"/>
-      <c r="AB3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n"/>
@@ -1256,26 +1092,6 @@
       <c r="F4" s="7" t="n"/>
       <c r="G4" s="7" t="n"/>
       <c r="H4" s="7" t="n"/>
-      <c r="I4" s="7" t="n"/>
-      <c r="J4" s="7" t="n"/>
-      <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="n"/>
-      <c r="M4" s="7" t="n"/>
-      <c r="N4" s="7" t="n"/>
-      <c r="O4" s="7" t="n"/>
-      <c r="P4" s="7" t="n"/>
-      <c r="Q4" s="7" t="n"/>
-      <c r="R4" s="7" t="n"/>
-      <c r="S4" s="7" t="n"/>
-      <c r="T4" s="7" t="n"/>
-      <c r="U4" s="7" t="n"/>
-      <c r="V4" s="7" t="n"/>
-      <c r="W4" s="7" t="n"/>
-      <c r="X4" s="7" t="n"/>
-      <c r="Y4" s="7" t="n"/>
-      <c r="Z4" s="7" t="n"/>
-      <c r="AA4" s="7" t="n"/>
-      <c r="AB4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n"/>
@@ -1286,26 +1102,6 @@
       <c r="F5" s="7" t="n"/>
       <c r="G5" s="7" t="n"/>
       <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
-      <c r="M5" s="7" t="n"/>
-      <c r="N5" s="7" t="n"/>
-      <c r="O5" s="7" t="n"/>
-      <c r="P5" s="7" t="n"/>
-      <c r="Q5" s="7" t="n"/>
-      <c r="R5" s="7" t="n"/>
-      <c r="S5" s="7" t="n"/>
-      <c r="T5" s="7" t="n"/>
-      <c r="U5" s="7" t="n"/>
-      <c r="V5" s="7" t="n"/>
-      <c r="W5" s="7" t="n"/>
-      <c r="X5" s="7" t="n"/>
-      <c r="Y5" s="7" t="n"/>
-      <c r="Z5" s="7" t="n"/>
-      <c r="AA5" s="7" t="n"/>
-      <c r="AB5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n"/>
@@ -1316,26 +1112,6 @@
       <c r="F6" s="7" t="n"/>
       <c r="G6" s="7" t="n"/>
       <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="7" t="n"/>
-      <c r="M6" s="7" t="n"/>
-      <c r="N6" s="7" t="n"/>
-      <c r="O6" s="7" t="n"/>
-      <c r="P6" s="7" t="n"/>
-      <c r="Q6" s="7" t="n"/>
-      <c r="R6" s="7" t="n"/>
-      <c r="S6" s="7" t="n"/>
-      <c r="T6" s="7" t="n"/>
-      <c r="U6" s="7" t="n"/>
-      <c r="V6" s="7" t="n"/>
-      <c r="W6" s="7" t="n"/>
-      <c r="X6" s="7" t="n"/>
-      <c r="Y6" s="7" t="n"/>
-      <c r="Z6" s="7" t="n"/>
-      <c r="AA6" s="7" t="n"/>
-      <c r="AB6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n"/>
@@ -1346,26 +1122,6 @@
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="7" t="n"/>
       <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
-      <c r="O7" s="7" t="n"/>
-      <c r="P7" s="7" t="n"/>
-      <c r="Q7" s="7" t="n"/>
-      <c r="R7" s="7" t="n"/>
-      <c r="S7" s="7" t="n"/>
-      <c r="T7" s="7" t="n"/>
-      <c r="U7" s="7" t="n"/>
-      <c r="V7" s="7" t="n"/>
-      <c r="W7" s="7" t="n"/>
-      <c r="X7" s="7" t="n"/>
-      <c r="Y7" s="7" t="n"/>
-      <c r="Z7" s="7" t="n"/>
-      <c r="AA7" s="7" t="n"/>
-      <c r="AB7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n"/>
@@ -1376,26 +1132,6 @@
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="7" t="n"/>
       <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="7" t="n"/>
-      <c r="M8" s="7" t="n"/>
-      <c r="N8" s="7" t="n"/>
-      <c r="O8" s="7" t="n"/>
-      <c r="P8" s="7" t="n"/>
-      <c r="Q8" s="7" t="n"/>
-      <c r="R8" s="7" t="n"/>
-      <c r="S8" s="7" t="n"/>
-      <c r="T8" s="7" t="n"/>
-      <c r="U8" s="7" t="n"/>
-      <c r="V8" s="7" t="n"/>
-      <c r="W8" s="7" t="n"/>
-      <c r="X8" s="7" t="n"/>
-      <c r="Y8" s="7" t="n"/>
-      <c r="Z8" s="7" t="n"/>
-      <c r="AA8" s="7" t="n"/>
-      <c r="AB8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n"/>
@@ -1406,26 +1142,6 @@
       <c r="F9" s="7" t="n"/>
       <c r="G9" s="7" t="n"/>
       <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
-      <c r="O9" s="7" t="n"/>
-      <c r="P9" s="7" t="n"/>
-      <c r="Q9" s="7" t="n"/>
-      <c r="R9" s="7" t="n"/>
-      <c r="S9" s="7" t="n"/>
-      <c r="T9" s="7" t="n"/>
-      <c r="U9" s="7" t="n"/>
-      <c r="V9" s="7" t="n"/>
-      <c r="W9" s="7" t="n"/>
-      <c r="X9" s="7" t="n"/>
-      <c r="Y9" s="7" t="n"/>
-      <c r="Z9" s="7" t="n"/>
-      <c r="AA9" s="7" t="n"/>
-      <c r="AB9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n"/>
@@ -1436,26 +1152,6 @@
       <c r="F10" s="7" t="n"/>
       <c r="G10" s="7" t="n"/>
       <c r="H10" s="7" t="n"/>
-      <c r="I10" s="7" t="n"/>
-      <c r="J10" s="7" t="n"/>
-      <c r="K10" s="7" t="n"/>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7" t="n"/>
-      <c r="N10" s="7" t="n"/>
-      <c r="O10" s="7" t="n"/>
-      <c r="P10" s="7" t="n"/>
-      <c r="Q10" s="7" t="n"/>
-      <c r="R10" s="7" t="n"/>
-      <c r="S10" s="7" t="n"/>
-      <c r="T10" s="7" t="n"/>
-      <c r="U10" s="7" t="n"/>
-      <c r="V10" s="7" t="n"/>
-      <c r="W10" s="7" t="n"/>
-      <c r="X10" s="7" t="n"/>
-      <c r="Y10" s="7" t="n"/>
-      <c r="Z10" s="7" t="n"/>
-      <c r="AA10" s="7" t="n"/>
-      <c r="AB10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -1466,26 +1162,6 @@
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="7" t="n"/>
       <c r="H11" s="7" t="n"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
-      <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7" t="n"/>
-      <c r="N11" s="7" t="n"/>
-      <c r="O11" s="7" t="n"/>
-      <c r="P11" s="7" t="n"/>
-      <c r="Q11" s="7" t="n"/>
-      <c r="R11" s="7" t="n"/>
-      <c r="S11" s="7" t="n"/>
-      <c r="T11" s="7" t="n"/>
-      <c r="U11" s="7" t="n"/>
-      <c r="V11" s="7" t="n"/>
-      <c r="W11" s="7" t="n"/>
-      <c r="X11" s="7" t="n"/>
-      <c r="Y11" s="7" t="n"/>
-      <c r="Z11" s="7" t="n"/>
-      <c r="AA11" s="7" t="n"/>
-      <c r="AB11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -1496,26 +1172,6 @@
       <c r="F12" s="7" t="n"/>
       <c r="G12" s="7" t="n"/>
       <c r="H12" s="7" t="n"/>
-      <c r="I12" s="7" t="n"/>
-      <c r="J12" s="7" t="n"/>
-      <c r="K12" s="7" t="n"/>
-      <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7" t="n"/>
-      <c r="N12" s="7" t="n"/>
-      <c r="O12" s="7" t="n"/>
-      <c r="P12" s="7" t="n"/>
-      <c r="Q12" s="7" t="n"/>
-      <c r="R12" s="7" t="n"/>
-      <c r="S12" s="7" t="n"/>
-      <c r="T12" s="7" t="n"/>
-      <c r="U12" s="7" t="n"/>
-      <c r="V12" s="7" t="n"/>
-      <c r="W12" s="7" t="n"/>
-      <c r="X12" s="7" t="n"/>
-      <c r="Y12" s="7" t="n"/>
-      <c r="Z12" s="7" t="n"/>
-      <c r="AA12" s="7" t="n"/>
-      <c r="AB12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
@@ -1526,26 +1182,6 @@
       <c r="F13" s="7" t="n"/>
       <c r="G13" s="7" t="n"/>
       <c r="H13" s="7" t="n"/>
-      <c r="I13" s="7" t="n"/>
-      <c r="J13" s="7" t="n"/>
-      <c r="K13" s="7" t="n"/>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7" t="n"/>
-      <c r="N13" s="7" t="n"/>
-      <c r="O13" s="7" t="n"/>
-      <c r="P13" s="7" t="n"/>
-      <c r="Q13" s="7" t="n"/>
-      <c r="R13" s="7" t="n"/>
-      <c r="S13" s="7" t="n"/>
-      <c r="T13" s="7" t="n"/>
-      <c r="U13" s="7" t="n"/>
-      <c r="V13" s="7" t="n"/>
-      <c r="W13" s="7" t="n"/>
-      <c r="X13" s="7" t="n"/>
-      <c r="Y13" s="7" t="n"/>
-      <c r="Z13" s="7" t="n"/>
-      <c r="AA13" s="7" t="n"/>
-      <c r="AB13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -1556,26 +1192,6 @@
       <c r="F14" s="7" t="n"/>
       <c r="G14" s="7" t="n"/>
       <c r="H14" s="7" t="n"/>
-      <c r="I14" s="7" t="n"/>
-      <c r="J14" s="7" t="n"/>
-      <c r="K14" s="7" t="n"/>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7" t="n"/>
-      <c r="N14" s="7" t="n"/>
-      <c r="O14" s="7" t="n"/>
-      <c r="P14" s="7" t="n"/>
-      <c r="Q14" s="7" t="n"/>
-      <c r="R14" s="7" t="n"/>
-      <c r="S14" s="7" t="n"/>
-      <c r="T14" s="7" t="n"/>
-      <c r="U14" s="7" t="n"/>
-      <c r="V14" s="7" t="n"/>
-      <c r="W14" s="7" t="n"/>
-      <c r="X14" s="7" t="n"/>
-      <c r="Y14" s="7" t="n"/>
-      <c r="Z14" s="7" t="n"/>
-      <c r="AA14" s="7" t="n"/>
-      <c r="AB14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -1586,26 +1202,6 @@
       <c r="F15" s="7" t="n"/>
       <c r="G15" s="7" t="n"/>
       <c r="H15" s="7" t="n"/>
-      <c r="I15" s="7" t="n"/>
-      <c r="J15" s="7" t="n"/>
-      <c r="K15" s="7" t="n"/>
-      <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7" t="n"/>
-      <c r="N15" s="7" t="n"/>
-      <c r="O15" s="7" t="n"/>
-      <c r="P15" s="7" t="n"/>
-      <c r="Q15" s="7" t="n"/>
-      <c r="R15" s="7" t="n"/>
-      <c r="S15" s="7" t="n"/>
-      <c r="T15" s="7" t="n"/>
-      <c r="U15" s="7" t="n"/>
-      <c r="V15" s="7" t="n"/>
-      <c r="W15" s="7" t="n"/>
-      <c r="X15" s="7" t="n"/>
-      <c r="Y15" s="7" t="n"/>
-      <c r="Z15" s="7" t="n"/>
-      <c r="AA15" s="7" t="n"/>
-      <c r="AB15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
@@ -1616,26 +1212,6 @@
       <c r="F16" s="7" t="n"/>
       <c r="G16" s="7" t="n"/>
       <c r="H16" s="7" t="n"/>
-      <c r="I16" s="7" t="n"/>
-      <c r="J16" s="7" t="n"/>
-      <c r="K16" s="7" t="n"/>
-      <c r="L16" s="7" t="n"/>
-      <c r="M16" s="7" t="n"/>
-      <c r="N16" s="7" t="n"/>
-      <c r="O16" s="7" t="n"/>
-      <c r="P16" s="7" t="n"/>
-      <c r="Q16" s="7" t="n"/>
-      <c r="R16" s="7" t="n"/>
-      <c r="S16" s="7" t="n"/>
-      <c r="T16" s="7" t="n"/>
-      <c r="U16" s="7" t="n"/>
-      <c r="V16" s="7" t="n"/>
-      <c r="W16" s="7" t="n"/>
-      <c r="X16" s="7" t="n"/>
-      <c r="Y16" s="7" t="n"/>
-      <c r="Z16" s="7" t="n"/>
-      <c r="AA16" s="7" t="n"/>
-      <c r="AB16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
@@ -1646,26 +1222,6 @@
       <c r="F17" s="7" t="n"/>
       <c r="G17" s="7" t="n"/>
       <c r="H17" s="7" t="n"/>
-      <c r="I17" s="7" t="n"/>
-      <c r="J17" s="7" t="n"/>
-      <c r="K17" s="7" t="n"/>
-      <c r="L17" s="7" t="n"/>
-      <c r="M17" s="7" t="n"/>
-      <c r="N17" s="7" t="n"/>
-      <c r="O17" s="7" t="n"/>
-      <c r="P17" s="7" t="n"/>
-      <c r="Q17" s="7" t="n"/>
-      <c r="R17" s="7" t="n"/>
-      <c r="S17" s="7" t="n"/>
-      <c r="T17" s="7" t="n"/>
-      <c r="U17" s="7" t="n"/>
-      <c r="V17" s="7" t="n"/>
-      <c r="W17" s="7" t="n"/>
-      <c r="X17" s="7" t="n"/>
-      <c r="Y17" s="7" t="n"/>
-      <c r="Z17" s="7" t="n"/>
-      <c r="AA17" s="7" t="n"/>
-      <c r="AB17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
@@ -1676,26 +1232,6 @@
       <c r="F18" s="7" t="n"/>
       <c r="G18" s="7" t="n"/>
       <c r="H18" s="7" t="n"/>
-      <c r="I18" s="7" t="n"/>
-      <c r="J18" s="7" t="n"/>
-      <c r="K18" s="7" t="n"/>
-      <c r="L18" s="7" t="n"/>
-      <c r="M18" s="7" t="n"/>
-      <c r="N18" s="7" t="n"/>
-      <c r="O18" s="7" t="n"/>
-      <c r="P18" s="7" t="n"/>
-      <c r="Q18" s="7" t="n"/>
-      <c r="R18" s="7" t="n"/>
-      <c r="S18" s="7" t="n"/>
-      <c r="T18" s="7" t="n"/>
-      <c r="U18" s="7" t="n"/>
-      <c r="V18" s="7" t="n"/>
-      <c r="W18" s="7" t="n"/>
-      <c r="X18" s="7" t="n"/>
-      <c r="Y18" s="7" t="n"/>
-      <c r="Z18" s="7" t="n"/>
-      <c r="AA18" s="7" t="n"/>
-      <c r="AB18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n"/>
@@ -1706,26 +1242,6 @@
       <c r="F19" s="7" t="n"/>
       <c r="G19" s="7" t="n"/>
       <c r="H19" s="7" t="n"/>
-      <c r="I19" s="7" t="n"/>
-      <c r="J19" s="7" t="n"/>
-      <c r="K19" s="7" t="n"/>
-      <c r="L19" s="7" t="n"/>
-      <c r="M19" s="7" t="n"/>
-      <c r="N19" s="7" t="n"/>
-      <c r="O19" s="7" t="n"/>
-      <c r="P19" s="7" t="n"/>
-      <c r="Q19" s="7" t="n"/>
-      <c r="R19" s="7" t="n"/>
-      <c r="S19" s="7" t="n"/>
-      <c r="T19" s="7" t="n"/>
-      <c r="U19" s="7" t="n"/>
-      <c r="V19" s="7" t="n"/>
-      <c r="W19" s="7" t="n"/>
-      <c r="X19" s="7" t="n"/>
-      <c r="Y19" s="7" t="n"/>
-      <c r="Z19" s="7" t="n"/>
-      <c r="AA19" s="7" t="n"/>
-      <c r="AB19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n"/>
@@ -1736,26 +1252,6 @@
       <c r="F20" s="7" t="n"/>
       <c r="G20" s="7" t="n"/>
       <c r="H20" s="7" t="n"/>
-      <c r="I20" s="7" t="n"/>
-      <c r="J20" s="7" t="n"/>
-      <c r="K20" s="7" t="n"/>
-      <c r="L20" s="7" t="n"/>
-      <c r="M20" s="7" t="n"/>
-      <c r="N20" s="7" t="n"/>
-      <c r="O20" s="7" t="n"/>
-      <c r="P20" s="7" t="n"/>
-      <c r="Q20" s="7" t="n"/>
-      <c r="R20" s="7" t="n"/>
-      <c r="S20" s="7" t="n"/>
-      <c r="T20" s="7" t="n"/>
-      <c r="U20" s="7" t="n"/>
-      <c r="V20" s="7" t="n"/>
-      <c r="W20" s="7" t="n"/>
-      <c r="X20" s="7" t="n"/>
-      <c r="Y20" s="7" t="n"/>
-      <c r="Z20" s="7" t="n"/>
-      <c r="AA20" s="7" t="n"/>
-      <c r="AB20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n"/>
@@ -1766,26 +1262,6 @@
       <c r="F21" s="7" t="n"/>
       <c r="G21" s="7" t="n"/>
       <c r="H21" s="7" t="n"/>
-      <c r="I21" s="7" t="n"/>
-      <c r="J21" s="7" t="n"/>
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
-      <c r="N21" s="7" t="n"/>
-      <c r="O21" s="7" t="n"/>
-      <c r="P21" s="7" t="n"/>
-      <c r="Q21" s="7" t="n"/>
-      <c r="R21" s="7" t="n"/>
-      <c r="S21" s="7" t="n"/>
-      <c r="T21" s="7" t="n"/>
-      <c r="U21" s="7" t="n"/>
-      <c r="V21" s="7" t="n"/>
-      <c r="W21" s="7" t="n"/>
-      <c r="X21" s="7" t="n"/>
-      <c r="Y21" s="7" t="n"/>
-      <c r="Z21" s="7" t="n"/>
-      <c r="AA21" s="7" t="n"/>
-      <c r="AB21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n"/>
@@ -1796,26 +1272,6 @@
       <c r="F22" s="7" t="n"/>
       <c r="G22" s="7" t="n"/>
       <c r="H22" s="7" t="n"/>
-      <c r="I22" s="7" t="n"/>
-      <c r="J22" s="7" t="n"/>
-      <c r="K22" s="7" t="n"/>
-      <c r="L22" s="7" t="n"/>
-      <c r="M22" s="7" t="n"/>
-      <c r="N22" s="7" t="n"/>
-      <c r="O22" s="7" t="n"/>
-      <c r="P22" s="7" t="n"/>
-      <c r="Q22" s="7" t="n"/>
-      <c r="R22" s="7" t="n"/>
-      <c r="S22" s="7" t="n"/>
-      <c r="T22" s="7" t="n"/>
-      <c r="U22" s="7" t="n"/>
-      <c r="V22" s="7" t="n"/>
-      <c r="W22" s="7" t="n"/>
-      <c r="X22" s="7" t="n"/>
-      <c r="Y22" s="7" t="n"/>
-      <c r="Z22" s="7" t="n"/>
-      <c r="AA22" s="7" t="n"/>
-      <c r="AB22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -1826,26 +1282,6 @@
       <c r="F23" s="7" t="n"/>
       <c r="G23" s="7" t="n"/>
       <c r="H23" s="7" t="n"/>
-      <c r="I23" s="7" t="n"/>
-      <c r="J23" s="7" t="n"/>
-      <c r="K23" s="7" t="n"/>
-      <c r="L23" s="7" t="n"/>
-      <c r="M23" s="7" t="n"/>
-      <c r="N23" s="7" t="n"/>
-      <c r="O23" s="7" t="n"/>
-      <c r="P23" s="7" t="n"/>
-      <c r="Q23" s="7" t="n"/>
-      <c r="R23" s="7" t="n"/>
-      <c r="S23" s="7" t="n"/>
-      <c r="T23" s="7" t="n"/>
-      <c r="U23" s="7" t="n"/>
-      <c r="V23" s="7" t="n"/>
-      <c r="W23" s="7" t="n"/>
-      <c r="X23" s="7" t="n"/>
-      <c r="Y23" s="7" t="n"/>
-      <c r="Z23" s="7" t="n"/>
-      <c r="AA23" s="7" t="n"/>
-      <c r="AB23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n"/>
@@ -1856,26 +1292,6 @@
       <c r="F24" s="7" t="n"/>
       <c r="G24" s="7" t="n"/>
       <c r="H24" s="7" t="n"/>
-      <c r="I24" s="7" t="n"/>
-      <c r="J24" s="7" t="n"/>
-      <c r="K24" s="7" t="n"/>
-      <c r="L24" s="7" t="n"/>
-      <c r="M24" s="7" t="n"/>
-      <c r="N24" s="7" t="n"/>
-      <c r="O24" s="7" t="n"/>
-      <c r="P24" s="7" t="n"/>
-      <c r="Q24" s="7" t="n"/>
-      <c r="R24" s="7" t="n"/>
-      <c r="S24" s="7" t="n"/>
-      <c r="T24" s="7" t="n"/>
-      <c r="U24" s="7" t="n"/>
-      <c r="V24" s="7" t="n"/>
-      <c r="W24" s="7" t="n"/>
-      <c r="X24" s="7" t="n"/>
-      <c r="Y24" s="7" t="n"/>
-      <c r="Z24" s="7" t="n"/>
-      <c r="AA24" s="7" t="n"/>
-      <c r="AB24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -1886,26 +1302,6 @@
       <c r="F25" s="7" t="n"/>
       <c r="G25" s="7" t="n"/>
       <c r="H25" s="7" t="n"/>
-      <c r="I25" s="7" t="n"/>
-      <c r="J25" s="7" t="n"/>
-      <c r="K25" s="7" t="n"/>
-      <c r="L25" s="7" t="n"/>
-      <c r="M25" s="7" t="n"/>
-      <c r="N25" s="7" t="n"/>
-      <c r="O25" s="7" t="n"/>
-      <c r="P25" s="7" t="n"/>
-      <c r="Q25" s="7" t="n"/>
-      <c r="R25" s="7" t="n"/>
-      <c r="S25" s="7" t="n"/>
-      <c r="T25" s="7" t="n"/>
-      <c r="U25" s="7" t="n"/>
-      <c r="V25" s="7" t="n"/>
-      <c r="W25" s="7" t="n"/>
-      <c r="X25" s="7" t="n"/>
-      <c r="Y25" s="7" t="n"/>
-      <c r="Z25" s="7" t="n"/>
-      <c r="AA25" s="7" t="n"/>
-      <c r="AB25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n"/>
@@ -1916,26 +1312,6 @@
       <c r="F26" s="7" t="n"/>
       <c r="G26" s="7" t="n"/>
       <c r="H26" s="7" t="n"/>
-      <c r="I26" s="7" t="n"/>
-      <c r="J26" s="7" t="n"/>
-      <c r="K26" s="7" t="n"/>
-      <c r="L26" s="7" t="n"/>
-      <c r="M26" s="7" t="n"/>
-      <c r="N26" s="7" t="n"/>
-      <c r="O26" s="7" t="n"/>
-      <c r="P26" s="7" t="n"/>
-      <c r="Q26" s="7" t="n"/>
-      <c r="R26" s="7" t="n"/>
-      <c r="S26" s="7" t="n"/>
-      <c r="T26" s="7" t="n"/>
-      <c r="U26" s="7" t="n"/>
-      <c r="V26" s="7" t="n"/>
-      <c r="W26" s="7" t="n"/>
-      <c r="X26" s="7" t="n"/>
-      <c r="Y26" s="7" t="n"/>
-      <c r="Z26" s="7" t="n"/>
-      <c r="AA26" s="7" t="n"/>
-      <c r="AB26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n"/>
@@ -1946,26 +1322,6 @@
       <c r="F27" s="7" t="n"/>
       <c r="G27" s="7" t="n"/>
       <c r="H27" s="7" t="n"/>
-      <c r="I27" s="7" t="n"/>
-      <c r="J27" s="7" t="n"/>
-      <c r="K27" s="7" t="n"/>
-      <c r="L27" s="7" t="n"/>
-      <c r="M27" s="7" t="n"/>
-      <c r="N27" s="7" t="n"/>
-      <c r="O27" s="7" t="n"/>
-      <c r="P27" s="7" t="n"/>
-      <c r="Q27" s="7" t="n"/>
-      <c r="R27" s="7" t="n"/>
-      <c r="S27" s="7" t="n"/>
-      <c r="T27" s="7" t="n"/>
-      <c r="U27" s="7" t="n"/>
-      <c r="V27" s="7" t="n"/>
-      <c r="W27" s="7" t="n"/>
-      <c r="X27" s="7" t="n"/>
-      <c r="Y27" s="7" t="n"/>
-      <c r="Z27" s="7" t="n"/>
-      <c r="AA27" s="7" t="n"/>
-      <c r="AB27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n"/>
@@ -1976,26 +1332,6 @@
       <c r="F28" s="7" t="n"/>
       <c r="G28" s="7" t="n"/>
       <c r="H28" s="7" t="n"/>
-      <c r="I28" s="7" t="n"/>
-      <c r="J28" s="7" t="n"/>
-      <c r="K28" s="7" t="n"/>
-      <c r="L28" s="7" t="n"/>
-      <c r="M28" s="7" t="n"/>
-      <c r="N28" s="7" t="n"/>
-      <c r="O28" s="7" t="n"/>
-      <c r="P28" s="7" t="n"/>
-      <c r="Q28" s="7" t="n"/>
-      <c r="R28" s="7" t="n"/>
-      <c r="S28" s="7" t="n"/>
-      <c r="T28" s="7" t="n"/>
-      <c r="U28" s="7" t="n"/>
-      <c r="V28" s="7" t="n"/>
-      <c r="W28" s="7" t="n"/>
-      <c r="X28" s="7" t="n"/>
-      <c r="Y28" s="7" t="n"/>
-      <c r="Z28" s="7" t="n"/>
-      <c r="AA28" s="7" t="n"/>
-      <c r="AB28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n"/>
@@ -2006,26 +1342,6 @@
       <c r="F29" s="7" t="n"/>
       <c r="G29" s="7" t="n"/>
       <c r="H29" s="7" t="n"/>
-      <c r="I29" s="7" t="n"/>
-      <c r="J29" s="7" t="n"/>
-      <c r="K29" s="7" t="n"/>
-      <c r="L29" s="7" t="n"/>
-      <c r="M29" s="7" t="n"/>
-      <c r="N29" s="7" t="n"/>
-      <c r="O29" s="7" t="n"/>
-      <c r="P29" s="7" t="n"/>
-      <c r="Q29" s="7" t="n"/>
-      <c r="R29" s="7" t="n"/>
-      <c r="S29" s="7" t="n"/>
-      <c r="T29" s="7" t="n"/>
-      <c r="U29" s="7" t="n"/>
-      <c r="V29" s="7" t="n"/>
-      <c r="W29" s="7" t="n"/>
-      <c r="X29" s="7" t="n"/>
-      <c r="Y29" s="7" t="n"/>
-      <c r="Z29" s="7" t="n"/>
-      <c r="AA29" s="7" t="n"/>
-      <c r="AB29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n"/>
@@ -2036,26 +1352,6 @@
       <c r="F30" s="7" t="n"/>
       <c r="G30" s="7" t="n"/>
       <c r="H30" s="7" t="n"/>
-      <c r="I30" s="7" t="n"/>
-      <c r="J30" s="7" t="n"/>
-      <c r="K30" s="7" t="n"/>
-      <c r="L30" s="7" t="n"/>
-      <c r="M30" s="7" t="n"/>
-      <c r="N30" s="7" t="n"/>
-      <c r="O30" s="7" t="n"/>
-      <c r="P30" s="7" t="n"/>
-      <c r="Q30" s="7" t="n"/>
-      <c r="R30" s="7" t="n"/>
-      <c r="S30" s="7" t="n"/>
-      <c r="T30" s="7" t="n"/>
-      <c r="U30" s="7" t="n"/>
-      <c r="V30" s="7" t="n"/>
-      <c r="W30" s="7" t="n"/>
-      <c r="X30" s="7" t="n"/>
-      <c r="Y30" s="7" t="n"/>
-      <c r="Z30" s="7" t="n"/>
-      <c r="AA30" s="7" t="n"/>
-      <c r="AB30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n"/>
@@ -2066,26 +1362,6 @@
       <c r="F31" s="7" t="n"/>
       <c r="G31" s="7" t="n"/>
       <c r="H31" s="7" t="n"/>
-      <c r="I31" s="7" t="n"/>
-      <c r="J31" s="7" t="n"/>
-      <c r="K31" s="7" t="n"/>
-      <c r="L31" s="7" t="n"/>
-      <c r="M31" s="7" t="n"/>
-      <c r="N31" s="7" t="n"/>
-      <c r="O31" s="7" t="n"/>
-      <c r="P31" s="7" t="n"/>
-      <c r="Q31" s="7" t="n"/>
-      <c r="R31" s="7" t="n"/>
-      <c r="S31" s="7" t="n"/>
-      <c r="T31" s="7" t="n"/>
-      <c r="U31" s="7" t="n"/>
-      <c r="V31" s="7" t="n"/>
-      <c r="W31" s="7" t="n"/>
-      <c r="X31" s="7" t="n"/>
-      <c r="Y31" s="7" t="n"/>
-      <c r="Z31" s="7" t="n"/>
-      <c r="AA31" s="7" t="n"/>
-      <c r="AB31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n"/>
@@ -2096,26 +1372,6 @@
       <c r="F32" s="7" t="n"/>
       <c r="G32" s="7" t="n"/>
       <c r="H32" s="7" t="n"/>
-      <c r="I32" s="7" t="n"/>
-      <c r="J32" s="7" t="n"/>
-      <c r="K32" s="7" t="n"/>
-      <c r="L32" s="7" t="n"/>
-      <c r="M32" s="7" t="n"/>
-      <c r="N32" s="7" t="n"/>
-      <c r="O32" s="7" t="n"/>
-      <c r="P32" s="7" t="n"/>
-      <c r="Q32" s="7" t="n"/>
-      <c r="R32" s="7" t="n"/>
-      <c r="S32" s="7" t="n"/>
-      <c r="T32" s="7" t="n"/>
-      <c r="U32" s="7" t="n"/>
-      <c r="V32" s="7" t="n"/>
-      <c r="W32" s="7" t="n"/>
-      <c r="X32" s="7" t="n"/>
-      <c r="Y32" s="7" t="n"/>
-      <c r="Z32" s="7" t="n"/>
-      <c r="AA32" s="7" t="n"/>
-      <c r="AB32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n"/>
@@ -2126,26 +1382,6 @@
       <c r="F33" s="7" t="n"/>
       <c r="G33" s="7" t="n"/>
       <c r="H33" s="7" t="n"/>
-      <c r="I33" s="7" t="n"/>
-      <c r="J33" s="7" t="n"/>
-      <c r="K33" s="7" t="n"/>
-      <c r="L33" s="7" t="n"/>
-      <c r="M33" s="7" t="n"/>
-      <c r="N33" s="7" t="n"/>
-      <c r="O33" s="7" t="n"/>
-      <c r="P33" s="7" t="n"/>
-      <c r="Q33" s="7" t="n"/>
-      <c r="R33" s="7" t="n"/>
-      <c r="S33" s="7" t="n"/>
-      <c r="T33" s="7" t="n"/>
-      <c r="U33" s="7" t="n"/>
-      <c r="V33" s="7" t="n"/>
-      <c r="W33" s="7" t="n"/>
-      <c r="X33" s="7" t="n"/>
-      <c r="Y33" s="7" t="n"/>
-      <c r="Z33" s="7" t="n"/>
-      <c r="AA33" s="7" t="n"/>
-      <c r="AB33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n"/>
@@ -2156,26 +1392,6 @@
       <c r="F34" s="7" t="n"/>
       <c r="G34" s="7" t="n"/>
       <c r="H34" s="7" t="n"/>
-      <c r="I34" s="7" t="n"/>
-      <c r="J34" s="7" t="n"/>
-      <c r="K34" s="7" t="n"/>
-      <c r="L34" s="7" t="n"/>
-      <c r="M34" s="7" t="n"/>
-      <c r="N34" s="7" t="n"/>
-      <c r="O34" s="7" t="n"/>
-      <c r="P34" s="7" t="n"/>
-      <c r="Q34" s="7" t="n"/>
-      <c r="R34" s="7" t="n"/>
-      <c r="S34" s="7" t="n"/>
-      <c r="T34" s="7" t="n"/>
-      <c r="U34" s="7" t="n"/>
-      <c r="V34" s="7" t="n"/>
-      <c r="W34" s="7" t="n"/>
-      <c r="X34" s="7" t="n"/>
-      <c r="Y34" s="7" t="n"/>
-      <c r="Z34" s="7" t="n"/>
-      <c r="AA34" s="7" t="n"/>
-      <c r="AB34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n"/>
@@ -2186,26 +1402,6 @@
       <c r="F35" s="7" t="n"/>
       <c r="G35" s="7" t="n"/>
       <c r="H35" s="7" t="n"/>
-      <c r="I35" s="7" t="n"/>
-      <c r="J35" s="7" t="n"/>
-      <c r="K35" s="7" t="n"/>
-      <c r="L35" s="7" t="n"/>
-      <c r="M35" s="7" t="n"/>
-      <c r="N35" s="7" t="n"/>
-      <c r="O35" s="7" t="n"/>
-      <c r="P35" s="7" t="n"/>
-      <c r="Q35" s="7" t="n"/>
-      <c r="R35" s="7" t="n"/>
-      <c r="S35" s="7" t="n"/>
-      <c r="T35" s="7" t="n"/>
-      <c r="U35" s="7" t="n"/>
-      <c r="V35" s="7" t="n"/>
-      <c r="W35" s="7" t="n"/>
-      <c r="X35" s="7" t="n"/>
-      <c r="Y35" s="7" t="n"/>
-      <c r="Z35" s="7" t="n"/>
-      <c r="AA35" s="7" t="n"/>
-      <c r="AB35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n"/>
@@ -2216,26 +1412,6 @@
       <c r="F36" s="7" t="n"/>
       <c r="G36" s="7" t="n"/>
       <c r="H36" s="7" t="n"/>
-      <c r="I36" s="7" t="n"/>
-      <c r="J36" s="7" t="n"/>
-      <c r="K36" s="7" t="n"/>
-      <c r="L36" s="7" t="n"/>
-      <c r="M36" s="7" t="n"/>
-      <c r="N36" s="7" t="n"/>
-      <c r="O36" s="7" t="n"/>
-      <c r="P36" s="7" t="n"/>
-      <c r="Q36" s="7" t="n"/>
-      <c r="R36" s="7" t="n"/>
-      <c r="S36" s="7" t="n"/>
-      <c r="T36" s="7" t="n"/>
-      <c r="U36" s="7" t="n"/>
-      <c r="V36" s="7" t="n"/>
-      <c r="W36" s="7" t="n"/>
-      <c r="X36" s="7" t="n"/>
-      <c r="Y36" s="7" t="n"/>
-      <c r="Z36" s="7" t="n"/>
-      <c r="AA36" s="7" t="n"/>
-      <c r="AB36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -2246,26 +1422,6 @@
       <c r="F37" s="7" t="n"/>
       <c r="G37" s="7" t="n"/>
       <c r="H37" s="7" t="n"/>
-      <c r="I37" s="7" t="n"/>
-      <c r="J37" s="7" t="n"/>
-      <c r="K37" s="7" t="n"/>
-      <c r="L37" s="7" t="n"/>
-      <c r="M37" s="7" t="n"/>
-      <c r="N37" s="7" t="n"/>
-      <c r="O37" s="7" t="n"/>
-      <c r="P37" s="7" t="n"/>
-      <c r="Q37" s="7" t="n"/>
-      <c r="R37" s="7" t="n"/>
-      <c r="S37" s="7" t="n"/>
-      <c r="T37" s="7" t="n"/>
-      <c r="U37" s="7" t="n"/>
-      <c r="V37" s="7" t="n"/>
-      <c r="W37" s="7" t="n"/>
-      <c r="X37" s="7" t="n"/>
-      <c r="Y37" s="7" t="n"/>
-      <c r="Z37" s="7" t="n"/>
-      <c r="AA37" s="7" t="n"/>
-      <c r="AB37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n"/>
@@ -2276,26 +1432,6 @@
       <c r="F38" s="7" t="n"/>
       <c r="G38" s="7" t="n"/>
       <c r="H38" s="7" t="n"/>
-      <c r="I38" s="7" t="n"/>
-      <c r="J38" s="7" t="n"/>
-      <c r="K38" s="7" t="n"/>
-      <c r="L38" s="7" t="n"/>
-      <c r="M38" s="7" t="n"/>
-      <c r="N38" s="7" t="n"/>
-      <c r="O38" s="7" t="n"/>
-      <c r="P38" s="7" t="n"/>
-      <c r="Q38" s="7" t="n"/>
-      <c r="R38" s="7" t="n"/>
-      <c r="S38" s="7" t="n"/>
-      <c r="T38" s="7" t="n"/>
-      <c r="U38" s="7" t="n"/>
-      <c r="V38" s="7" t="n"/>
-      <c r="W38" s="7" t="n"/>
-      <c r="X38" s="7" t="n"/>
-      <c r="Y38" s="7" t="n"/>
-      <c r="Z38" s="7" t="n"/>
-      <c r="AA38" s="7" t="n"/>
-      <c r="AB38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n"/>
@@ -2306,26 +1442,6 @@
       <c r="F39" s="7" t="n"/>
       <c r="G39" s="7" t="n"/>
       <c r="H39" s="7" t="n"/>
-      <c r="I39" s="7" t="n"/>
-      <c r="J39" s="7" t="n"/>
-      <c r="K39" s="7" t="n"/>
-      <c r="L39" s="7" t="n"/>
-      <c r="M39" s="7" t="n"/>
-      <c r="N39" s="7" t="n"/>
-      <c r="O39" s="7" t="n"/>
-      <c r="P39" s="7" t="n"/>
-      <c r="Q39" s="7" t="n"/>
-      <c r="R39" s="7" t="n"/>
-      <c r="S39" s="7" t="n"/>
-      <c r="T39" s="7" t="n"/>
-      <c r="U39" s="7" t="n"/>
-      <c r="V39" s="7" t="n"/>
-      <c r="W39" s="7" t="n"/>
-      <c r="X39" s="7" t="n"/>
-      <c r="Y39" s="7" t="n"/>
-      <c r="Z39" s="7" t="n"/>
-      <c r="AA39" s="7" t="n"/>
-      <c r="AB39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n"/>
@@ -2336,26 +1452,6 @@
       <c r="F40" s="7" t="n"/>
       <c r="G40" s="7" t="n"/>
       <c r="H40" s="7" t="n"/>
-      <c r="I40" s="7" t="n"/>
-      <c r="J40" s="7" t="n"/>
-      <c r="K40" s="7" t="n"/>
-      <c r="L40" s="7" t="n"/>
-      <c r="M40" s="7" t="n"/>
-      <c r="N40" s="7" t="n"/>
-      <c r="O40" s="7" t="n"/>
-      <c r="P40" s="7" t="n"/>
-      <c r="Q40" s="7" t="n"/>
-      <c r="R40" s="7" t="n"/>
-      <c r="S40" s="7" t="n"/>
-      <c r="T40" s="7" t="n"/>
-      <c r="U40" s="7" t="n"/>
-      <c r="V40" s="7" t="n"/>
-      <c r="W40" s="7" t="n"/>
-      <c r="X40" s="7" t="n"/>
-      <c r="Y40" s="7" t="n"/>
-      <c r="Z40" s="7" t="n"/>
-      <c r="AA40" s="7" t="n"/>
-      <c r="AB40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n"/>
@@ -2366,26 +1462,6 @@
       <c r="F41" s="7" t="n"/>
       <c r="G41" s="7" t="n"/>
       <c r="H41" s="7" t="n"/>
-      <c r="I41" s="7" t="n"/>
-      <c r="J41" s="7" t="n"/>
-      <c r="K41" s="7" t="n"/>
-      <c r="L41" s="7" t="n"/>
-      <c r="M41" s="7" t="n"/>
-      <c r="N41" s="7" t="n"/>
-      <c r="O41" s="7" t="n"/>
-      <c r="P41" s="7" t="n"/>
-      <c r="Q41" s="7" t="n"/>
-      <c r="R41" s="7" t="n"/>
-      <c r="S41" s="7" t="n"/>
-      <c r="T41" s="7" t="n"/>
-      <c r="U41" s="7" t="n"/>
-      <c r="V41" s="7" t="n"/>
-      <c r="W41" s="7" t="n"/>
-      <c r="X41" s="7" t="n"/>
-      <c r="Y41" s="7" t="n"/>
-      <c r="Z41" s="7" t="n"/>
-      <c r="AA41" s="7" t="n"/>
-      <c r="AB41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n"/>
@@ -2396,26 +1472,6 @@
       <c r="F42" s="7" t="n"/>
       <c r="G42" s="7" t="n"/>
       <c r="H42" s="7" t="n"/>
-      <c r="I42" s="7" t="n"/>
-      <c r="J42" s="7" t="n"/>
-      <c r="K42" s="7" t="n"/>
-      <c r="L42" s="7" t="n"/>
-      <c r="M42" s="7" t="n"/>
-      <c r="N42" s="7" t="n"/>
-      <c r="O42" s="7" t="n"/>
-      <c r="P42" s="7" t="n"/>
-      <c r="Q42" s="7" t="n"/>
-      <c r="R42" s="7" t="n"/>
-      <c r="S42" s="7" t="n"/>
-      <c r="T42" s="7" t="n"/>
-      <c r="U42" s="7" t="n"/>
-      <c r="V42" s="7" t="n"/>
-      <c r="W42" s="7" t="n"/>
-      <c r="X42" s="7" t="n"/>
-      <c r="Y42" s="7" t="n"/>
-      <c r="Z42" s="7" t="n"/>
-      <c r="AA42" s="7" t="n"/>
-      <c r="AB42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n"/>
@@ -2426,26 +1482,6 @@
       <c r="F43" s="7" t="n"/>
       <c r="G43" s="7" t="n"/>
       <c r="H43" s="7" t="n"/>
-      <c r="I43" s="7" t="n"/>
-      <c r="J43" s="7" t="n"/>
-      <c r="K43" s="7" t="n"/>
-      <c r="L43" s="7" t="n"/>
-      <c r="M43" s="7" t="n"/>
-      <c r="N43" s="7" t="n"/>
-      <c r="O43" s="7" t="n"/>
-      <c r="P43" s="7" t="n"/>
-      <c r="Q43" s="7" t="n"/>
-      <c r="R43" s="7" t="n"/>
-      <c r="S43" s="7" t="n"/>
-      <c r="T43" s="7" t="n"/>
-      <c r="U43" s="7" t="n"/>
-      <c r="V43" s="7" t="n"/>
-      <c r="W43" s="7" t="n"/>
-      <c r="X43" s="7" t="n"/>
-      <c r="Y43" s="7" t="n"/>
-      <c r="Z43" s="7" t="n"/>
-      <c r="AA43" s="7" t="n"/>
-      <c r="AB43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n"/>
@@ -2456,26 +1492,6 @@
       <c r="F44" s="7" t="n"/>
       <c r="G44" s="7" t="n"/>
       <c r="H44" s="7" t="n"/>
-      <c r="I44" s="7" t="n"/>
-      <c r="J44" s="7" t="n"/>
-      <c r="K44" s="7" t="n"/>
-      <c r="L44" s="7" t="n"/>
-      <c r="M44" s="7" t="n"/>
-      <c r="N44" s="7" t="n"/>
-      <c r="O44" s="7" t="n"/>
-      <c r="P44" s="7" t="n"/>
-      <c r="Q44" s="7" t="n"/>
-      <c r="R44" s="7" t="n"/>
-      <c r="S44" s="7" t="n"/>
-      <c r="T44" s="7" t="n"/>
-      <c r="U44" s="7" t="n"/>
-      <c r="V44" s="7" t="n"/>
-      <c r="W44" s="7" t="n"/>
-      <c r="X44" s="7" t="n"/>
-      <c r="Y44" s="7" t="n"/>
-      <c r="Z44" s="7" t="n"/>
-      <c r="AA44" s="7" t="n"/>
-      <c r="AB44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n"/>
@@ -2486,26 +1502,6 @@
       <c r="F45" s="7" t="n"/>
       <c r="G45" s="7" t="n"/>
       <c r="H45" s="7" t="n"/>
-      <c r="I45" s="7" t="n"/>
-      <c r="J45" s="7" t="n"/>
-      <c r="K45" s="7" t="n"/>
-      <c r="L45" s="7" t="n"/>
-      <c r="M45" s="7" t="n"/>
-      <c r="N45" s="7" t="n"/>
-      <c r="O45" s="7" t="n"/>
-      <c r="P45" s="7" t="n"/>
-      <c r="Q45" s="7" t="n"/>
-      <c r="R45" s="7" t="n"/>
-      <c r="S45" s="7" t="n"/>
-      <c r="T45" s="7" t="n"/>
-      <c r="U45" s="7" t="n"/>
-      <c r="V45" s="7" t="n"/>
-      <c r="W45" s="7" t="n"/>
-      <c r="X45" s="7" t="n"/>
-      <c r="Y45" s="7" t="n"/>
-      <c r="Z45" s="7" t="n"/>
-      <c r="AA45" s="7" t="n"/>
-      <c r="AB45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n"/>
@@ -2516,26 +1512,6 @@
       <c r="F46" s="7" t="n"/>
       <c r="G46" s="7" t="n"/>
       <c r="H46" s="7" t="n"/>
-      <c r="I46" s="7" t="n"/>
-      <c r="J46" s="7" t="n"/>
-      <c r="K46" s="7" t="n"/>
-      <c r="L46" s="7" t="n"/>
-      <c r="M46" s="7" t="n"/>
-      <c r="N46" s="7" t="n"/>
-      <c r="O46" s="7" t="n"/>
-      <c r="P46" s="7" t="n"/>
-      <c r="Q46" s="7" t="n"/>
-      <c r="R46" s="7" t="n"/>
-      <c r="S46" s="7" t="n"/>
-      <c r="T46" s="7" t="n"/>
-      <c r="U46" s="7" t="n"/>
-      <c r="V46" s="7" t="n"/>
-      <c r="W46" s="7" t="n"/>
-      <c r="X46" s="7" t="n"/>
-      <c r="Y46" s="7" t="n"/>
-      <c r="Z46" s="7" t="n"/>
-      <c r="AA46" s="7" t="n"/>
-      <c r="AB46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n"/>
@@ -2546,26 +1522,6 @@
       <c r="F47" s="7" t="n"/>
       <c r="G47" s="7" t="n"/>
       <c r="H47" s="7" t="n"/>
-      <c r="I47" s="7" t="n"/>
-      <c r="J47" s="7" t="n"/>
-      <c r="K47" s="7" t="n"/>
-      <c r="L47" s="7" t="n"/>
-      <c r="M47" s="7" t="n"/>
-      <c r="N47" s="7" t="n"/>
-      <c r="O47" s="7" t="n"/>
-      <c r="P47" s="7" t="n"/>
-      <c r="Q47" s="7" t="n"/>
-      <c r="R47" s="7" t="n"/>
-      <c r="S47" s="7" t="n"/>
-      <c r="T47" s="7" t="n"/>
-      <c r="U47" s="7" t="n"/>
-      <c r="V47" s="7" t="n"/>
-      <c r="W47" s="7" t="n"/>
-      <c r="X47" s="7" t="n"/>
-      <c r="Y47" s="7" t="n"/>
-      <c r="Z47" s="7" t="n"/>
-      <c r="AA47" s="7" t="n"/>
-      <c r="AB47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n"/>
@@ -2576,26 +1532,6 @@
       <c r="F48" s="7" t="n"/>
       <c r="G48" s="7" t="n"/>
       <c r="H48" s="7" t="n"/>
-      <c r="I48" s="7" t="n"/>
-      <c r="J48" s="7" t="n"/>
-      <c r="K48" s="7" t="n"/>
-      <c r="L48" s="7" t="n"/>
-      <c r="M48" s="7" t="n"/>
-      <c r="N48" s="7" t="n"/>
-      <c r="O48" s="7" t="n"/>
-      <c r="P48" s="7" t="n"/>
-      <c r="Q48" s="7" t="n"/>
-      <c r="R48" s="7" t="n"/>
-      <c r="S48" s="7" t="n"/>
-      <c r="T48" s="7" t="n"/>
-      <c r="U48" s="7" t="n"/>
-      <c r="V48" s="7" t="n"/>
-      <c r="W48" s="7" t="n"/>
-      <c r="X48" s="7" t="n"/>
-      <c r="Y48" s="7" t="n"/>
-      <c r="Z48" s="7" t="n"/>
-      <c r="AA48" s="7" t="n"/>
-      <c r="AB48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="n"/>
@@ -2606,26 +1542,6 @@
       <c r="F49" s="7" t="n"/>
       <c r="G49" s="7" t="n"/>
       <c r="H49" s="7" t="n"/>
-      <c r="I49" s="7" t="n"/>
-      <c r="J49" s="7" t="n"/>
-      <c r="K49" s="7" t="n"/>
-      <c r="L49" s="7" t="n"/>
-      <c r="M49" s="7" t="n"/>
-      <c r="N49" s="7" t="n"/>
-      <c r="O49" s="7" t="n"/>
-      <c r="P49" s="7" t="n"/>
-      <c r="Q49" s="7" t="n"/>
-      <c r="R49" s="7" t="n"/>
-      <c r="S49" s="7" t="n"/>
-      <c r="T49" s="7" t="n"/>
-      <c r="U49" s="7" t="n"/>
-      <c r="V49" s="7" t="n"/>
-      <c r="W49" s="7" t="n"/>
-      <c r="X49" s="7" t="n"/>
-      <c r="Y49" s="7" t="n"/>
-      <c r="Z49" s="7" t="n"/>
-      <c r="AA49" s="7" t="n"/>
-      <c r="AB49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n"/>
@@ -2636,26 +1552,6 @@
       <c r="F50" s="7" t="n"/>
       <c r="G50" s="7" t="n"/>
       <c r="H50" s="7" t="n"/>
-      <c r="I50" s="7" t="n"/>
-      <c r="J50" s="7" t="n"/>
-      <c r="K50" s="7" t="n"/>
-      <c r="L50" s="7" t="n"/>
-      <c r="M50" s="7" t="n"/>
-      <c r="N50" s="7" t="n"/>
-      <c r="O50" s="7" t="n"/>
-      <c r="P50" s="7" t="n"/>
-      <c r="Q50" s="7" t="n"/>
-      <c r="R50" s="7" t="n"/>
-      <c r="S50" s="7" t="n"/>
-      <c r="T50" s="7" t="n"/>
-      <c r="U50" s="7" t="n"/>
-      <c r="V50" s="7" t="n"/>
-      <c r="W50" s="7" t="n"/>
-      <c r="X50" s="7" t="n"/>
-      <c r="Y50" s="7" t="n"/>
-      <c r="Z50" s="7" t="n"/>
-      <c r="AA50" s="7" t="n"/>
-      <c r="AB50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="n"/>
@@ -2666,26 +1562,6 @@
       <c r="F51" s="7" t="n"/>
       <c r="G51" s="7" t="n"/>
       <c r="H51" s="7" t="n"/>
-      <c r="I51" s="7" t="n"/>
-      <c r="J51" s="7" t="n"/>
-      <c r="K51" s="7" t="n"/>
-      <c r="L51" s="7" t="n"/>
-      <c r="M51" s="7" t="n"/>
-      <c r="N51" s="7" t="n"/>
-      <c r="O51" s="7" t="n"/>
-      <c r="P51" s="7" t="n"/>
-      <c r="Q51" s="7" t="n"/>
-      <c r="R51" s="7" t="n"/>
-      <c r="S51" s="7" t="n"/>
-      <c r="T51" s="7" t="n"/>
-      <c r="U51" s="7" t="n"/>
-      <c r="V51" s="7" t="n"/>
-      <c r="W51" s="7" t="n"/>
-      <c r="X51" s="7" t="n"/>
-      <c r="Y51" s="7" t="n"/>
-      <c r="Z51" s="7" t="n"/>
-      <c r="AA51" s="7" t="n"/>
-      <c r="AB51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n"/>
@@ -2696,26 +1572,6 @@
       <c r="F52" s="7" t="n"/>
       <c r="G52" s="7" t="n"/>
       <c r="H52" s="7" t="n"/>
-      <c r="I52" s="7" t="n"/>
-      <c r="J52" s="7" t="n"/>
-      <c r="K52" s="7" t="n"/>
-      <c r="L52" s="7" t="n"/>
-      <c r="M52" s="7" t="n"/>
-      <c r="N52" s="7" t="n"/>
-      <c r="O52" s="7" t="n"/>
-      <c r="P52" s="7" t="n"/>
-      <c r="Q52" s="7" t="n"/>
-      <c r="R52" s="7" t="n"/>
-      <c r="S52" s="7" t="n"/>
-      <c r="T52" s="7" t="n"/>
-      <c r="U52" s="7" t="n"/>
-      <c r="V52" s="7" t="n"/>
-      <c r="W52" s="7" t="n"/>
-      <c r="X52" s="7" t="n"/>
-      <c r="Y52" s="7" t="n"/>
-      <c r="Z52" s="7" t="n"/>
-      <c r="AA52" s="7" t="n"/>
-      <c r="AB52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="n"/>
@@ -2726,26 +1582,6 @@
       <c r="F53" s="7" t="n"/>
       <c r="G53" s="7" t="n"/>
       <c r="H53" s="7" t="n"/>
-      <c r="I53" s="7" t="n"/>
-      <c r="J53" s="7" t="n"/>
-      <c r="K53" s="7" t="n"/>
-      <c r="L53" s="7" t="n"/>
-      <c r="M53" s="7" t="n"/>
-      <c r="N53" s="7" t="n"/>
-      <c r="O53" s="7" t="n"/>
-      <c r="P53" s="7" t="n"/>
-      <c r="Q53" s="7" t="n"/>
-      <c r="R53" s="7" t="n"/>
-      <c r="S53" s="7" t="n"/>
-      <c r="T53" s="7" t="n"/>
-      <c r="U53" s="7" t="n"/>
-      <c r="V53" s="7" t="n"/>
-      <c r="W53" s="7" t="n"/>
-      <c r="X53" s="7" t="n"/>
-      <c r="Y53" s="7" t="n"/>
-      <c r="Z53" s="7" t="n"/>
-      <c r="AA53" s="7" t="n"/>
-      <c r="AB53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n"/>
@@ -2756,26 +1592,6 @@
       <c r="F54" s="7" t="n"/>
       <c r="G54" s="7" t="n"/>
       <c r="H54" s="7" t="n"/>
-      <c r="I54" s="7" t="n"/>
-      <c r="J54" s="7" t="n"/>
-      <c r="K54" s="7" t="n"/>
-      <c r="L54" s="7" t="n"/>
-      <c r="M54" s="7" t="n"/>
-      <c r="N54" s="7" t="n"/>
-      <c r="O54" s="7" t="n"/>
-      <c r="P54" s="7" t="n"/>
-      <c r="Q54" s="7" t="n"/>
-      <c r="R54" s="7" t="n"/>
-      <c r="S54" s="7" t="n"/>
-      <c r="T54" s="7" t="n"/>
-      <c r="U54" s="7" t="n"/>
-      <c r="V54" s="7" t="n"/>
-      <c r="W54" s="7" t="n"/>
-      <c r="X54" s="7" t="n"/>
-      <c r="Y54" s="7" t="n"/>
-      <c r="Z54" s="7" t="n"/>
-      <c r="AA54" s="7" t="n"/>
-      <c r="AB54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="n"/>
@@ -2786,26 +1602,6 @@
       <c r="F55" s="7" t="n"/>
       <c r="G55" s="7" t="n"/>
       <c r="H55" s="7" t="n"/>
-      <c r="I55" s="7" t="n"/>
-      <c r="J55" s="7" t="n"/>
-      <c r="K55" s="7" t="n"/>
-      <c r="L55" s="7" t="n"/>
-      <c r="M55" s="7" t="n"/>
-      <c r="N55" s="7" t="n"/>
-      <c r="O55" s="7" t="n"/>
-      <c r="P55" s="7" t="n"/>
-      <c r="Q55" s="7" t="n"/>
-      <c r="R55" s="7" t="n"/>
-      <c r="S55" s="7" t="n"/>
-      <c r="T55" s="7" t="n"/>
-      <c r="U55" s="7" t="n"/>
-      <c r="V55" s="7" t="n"/>
-      <c r="W55" s="7" t="n"/>
-      <c r="X55" s="7" t="n"/>
-      <c r="Y55" s="7" t="n"/>
-      <c r="Z55" s="7" t="n"/>
-      <c r="AA55" s="7" t="n"/>
-      <c r="AB55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n"/>
@@ -2816,26 +1612,6 @@
       <c r="F56" s="7" t="n"/>
       <c r="G56" s="7" t="n"/>
       <c r="H56" s="7" t="n"/>
-      <c r="I56" s="7" t="n"/>
-      <c r="J56" s="7" t="n"/>
-      <c r="K56" s="7" t="n"/>
-      <c r="L56" s="7" t="n"/>
-      <c r="M56" s="7" t="n"/>
-      <c r="N56" s="7" t="n"/>
-      <c r="O56" s="7" t="n"/>
-      <c r="P56" s="7" t="n"/>
-      <c r="Q56" s="7" t="n"/>
-      <c r="R56" s="7" t="n"/>
-      <c r="S56" s="7" t="n"/>
-      <c r="T56" s="7" t="n"/>
-      <c r="U56" s="7" t="n"/>
-      <c r="V56" s="7" t="n"/>
-      <c r="W56" s="7" t="n"/>
-      <c r="X56" s="7" t="n"/>
-      <c r="Y56" s="7" t="n"/>
-      <c r="Z56" s="7" t="n"/>
-      <c r="AA56" s="7" t="n"/>
-      <c r="AB56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="n"/>
@@ -2846,26 +1622,6 @@
       <c r="F57" s="7" t="n"/>
       <c r="G57" s="7" t="n"/>
       <c r="H57" s="7" t="n"/>
-      <c r="I57" s="7" t="n"/>
-      <c r="J57" s="7" t="n"/>
-      <c r="K57" s="7" t="n"/>
-      <c r="L57" s="7" t="n"/>
-      <c r="M57" s="7" t="n"/>
-      <c r="N57" s="7" t="n"/>
-      <c r="O57" s="7" t="n"/>
-      <c r="P57" s="7" t="n"/>
-      <c r="Q57" s="7" t="n"/>
-      <c r="R57" s="7" t="n"/>
-      <c r="S57" s="7" t="n"/>
-      <c r="T57" s="7" t="n"/>
-      <c r="U57" s="7" t="n"/>
-      <c r="V57" s="7" t="n"/>
-      <c r="W57" s="7" t="n"/>
-      <c r="X57" s="7" t="n"/>
-      <c r="Y57" s="7" t="n"/>
-      <c r="Z57" s="7" t="n"/>
-      <c r="AA57" s="7" t="n"/>
-      <c r="AB57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n"/>
@@ -2876,26 +1632,6 @@
       <c r="F58" s="7" t="n"/>
       <c r="G58" s="7" t="n"/>
       <c r="H58" s="7" t="n"/>
-      <c r="I58" s="7" t="n"/>
-      <c r="J58" s="7" t="n"/>
-      <c r="K58" s="7" t="n"/>
-      <c r="L58" s="7" t="n"/>
-      <c r="M58" s="7" t="n"/>
-      <c r="N58" s="7" t="n"/>
-      <c r="O58" s="7" t="n"/>
-      <c r="P58" s="7" t="n"/>
-      <c r="Q58" s="7" t="n"/>
-      <c r="R58" s="7" t="n"/>
-      <c r="S58" s="7" t="n"/>
-      <c r="T58" s="7" t="n"/>
-      <c r="U58" s="7" t="n"/>
-      <c r="V58" s="7" t="n"/>
-      <c r="W58" s="7" t="n"/>
-      <c r="X58" s="7" t="n"/>
-      <c r="Y58" s="7" t="n"/>
-      <c r="Z58" s="7" t="n"/>
-      <c r="AA58" s="7" t="n"/>
-      <c r="AB58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="n"/>
@@ -2906,26 +1642,6 @@
       <c r="F59" s="7" t="n"/>
       <c r="G59" s="7" t="n"/>
       <c r="H59" s="7" t="n"/>
-      <c r="I59" s="7" t="n"/>
-      <c r="J59" s="7" t="n"/>
-      <c r="K59" s="7" t="n"/>
-      <c r="L59" s="7" t="n"/>
-      <c r="M59" s="7" t="n"/>
-      <c r="N59" s="7" t="n"/>
-      <c r="O59" s="7" t="n"/>
-      <c r="P59" s="7" t="n"/>
-      <c r="Q59" s="7" t="n"/>
-      <c r="R59" s="7" t="n"/>
-      <c r="S59" s="7" t="n"/>
-      <c r="T59" s="7" t="n"/>
-      <c r="U59" s="7" t="n"/>
-      <c r="V59" s="7" t="n"/>
-      <c r="W59" s="7" t="n"/>
-      <c r="X59" s="7" t="n"/>
-      <c r="Y59" s="7" t="n"/>
-      <c r="Z59" s="7" t="n"/>
-      <c r="AA59" s="7" t="n"/>
-      <c r="AB59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n"/>
@@ -2936,31 +1652,11 @@
       <c r="F60" s="7" t="n"/>
       <c r="G60" s="7" t="n"/>
       <c r="H60" s="7" t="n"/>
-      <c r="I60" s="7" t="n"/>
-      <c r="J60" s="7" t="n"/>
-      <c r="K60" s="7" t="n"/>
-      <c r="L60" s="7" t="n"/>
-      <c r="M60" s="7" t="n"/>
-      <c r="N60" s="7" t="n"/>
-      <c r="O60" s="7" t="n"/>
-      <c r="P60" s="7" t="n"/>
-      <c r="Q60" s="7" t="n"/>
-      <c r="R60" s="7" t="n"/>
-      <c r="S60" s="7" t="n"/>
-      <c r="T60" s="7" t="n"/>
-      <c r="U60" s="7" t="n"/>
-      <c r="V60" s="7" t="n"/>
-      <c r="W60" s="7" t="n"/>
-      <c r="X60" s="7" t="n"/>
-      <c r="Y60" s="7" t="n"/>
-      <c r="Z60" s="7" t="n"/>
-      <c r="AA60" s="7" t="n"/>
-      <c r="AB60" s="7" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="N2:N3000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$A$1:$A$4</formula1>
+    <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
+      <formula1>='Categories'!$A$3:$A$1000</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3316,10 +2012,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1001"/>
+  <dimension ref="A1:J1001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
@@ -3328,20 +2024,18 @@
     <col width="36" customWidth="1" min="7" max="7"/>
     <col width="31" customWidth="1" min="8" max="8"/>
     <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Category (pick)</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>Collection (as on the Collections sheet) *</t>
+          <t>Collection (pick from the Collections sheet) *</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
@@ -3366,7 +2060,7 @@
       </c>
       <c r="G1" s="8" t="inlineStr">
         <is>
-          <t>Warehouse (as on the Warehouses sheet)</t>
+          <t>Warehouse (pick from the Warehouses sheet)</t>
         </is>
       </c>
       <c r="H1" s="8" t="inlineStr">
@@ -3380,16 +2074,6 @@
         </is>
       </c>
       <c r="J1" s="8" t="inlineStr">
-        <is>
-          <t>Warn below (boxes)</t>
-        </is>
-      </c>
-      <c r="K1" s="8" t="inlineStr">
-        <is>
-          <t>Photo link</t>
-        </is>
-      </c>
-      <c r="L1" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -3434,11 +2118,7 @@
         <f>IF(OR(H2="",B2=""),"",IFERROR(ROUND(H2*MAX(VLOOKUP(B2,Collections!$B:$D,2,FALSE),VLOOKUP(B2,Collections!$B:$D,3,FALSE)*10.7639),0),"collection not found"))</f>
         <v/>
       </c>
-      <c r="J2" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="K2" s="6" t="inlineStr"/>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -3458,8 +2138,6 @@
         <v/>
       </c>
       <c r="J3" s="7" t="n"/>
-      <c r="K3" s="7" t="n"/>
-      <c r="L3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n"/>
@@ -3475,8 +2153,6 @@
         <v/>
       </c>
       <c r="J4" s="7" t="n"/>
-      <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n"/>
@@ -3492,8 +2168,6 @@
         <v/>
       </c>
       <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n"/>
@@ -3509,8 +2183,6 @@
         <v/>
       </c>
       <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n"/>
@@ -3526,8 +2198,6 @@
         <v/>
       </c>
       <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n"/>
@@ -3543,8 +2213,6 @@
         <v/>
       </c>
       <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n"/>
@@ -3560,8 +2228,6 @@
         <v/>
       </c>
       <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n"/>
@@ -3577,8 +2243,6 @@
         <v/>
       </c>
       <c r="J10" s="7" t="n"/>
-      <c r="K10" s="7" t="n"/>
-      <c r="L10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -3594,8 +2258,6 @@
         <v/>
       </c>
       <c r="J11" s="7" t="n"/>
-      <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -3611,8 +2273,6 @@
         <v/>
       </c>
       <c r="J12" s="7" t="n"/>
-      <c r="K12" s="7" t="n"/>
-      <c r="L12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
@@ -3628,8 +2288,6 @@
         <v/>
       </c>
       <c r="J13" s="7" t="n"/>
-      <c r="K13" s="7" t="n"/>
-      <c r="L13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -3645,8 +2303,6 @@
         <v/>
       </c>
       <c r="J14" s="7" t="n"/>
-      <c r="K14" s="7" t="n"/>
-      <c r="L14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -3662,8 +2318,6 @@
         <v/>
       </c>
       <c r="J15" s="7" t="n"/>
-      <c r="K15" s="7" t="n"/>
-      <c r="L15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
@@ -3679,8 +2333,6 @@
         <v/>
       </c>
       <c r="J16" s="7" t="n"/>
-      <c r="K16" s="7" t="n"/>
-      <c r="L16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
@@ -3696,8 +2348,6 @@
         <v/>
       </c>
       <c r="J17" s="7" t="n"/>
-      <c r="K17" s="7" t="n"/>
-      <c r="L17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
@@ -3713,8 +2363,6 @@
         <v/>
       </c>
       <c r="J18" s="7" t="n"/>
-      <c r="K18" s="7" t="n"/>
-      <c r="L18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n"/>
@@ -3730,8 +2378,6 @@
         <v/>
       </c>
       <c r="J19" s="7" t="n"/>
-      <c r="K19" s="7" t="n"/>
-      <c r="L19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n"/>
@@ -3747,8 +2393,6 @@
         <v/>
       </c>
       <c r="J20" s="7" t="n"/>
-      <c r="K20" s="7" t="n"/>
-      <c r="L20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n"/>
@@ -3764,8 +2408,6 @@
         <v/>
       </c>
       <c r="J21" s="7" t="n"/>
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n"/>
@@ -3781,8 +2423,6 @@
         <v/>
       </c>
       <c r="J22" s="7" t="n"/>
-      <c r="K22" s="7" t="n"/>
-      <c r="L22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -3798,8 +2438,6 @@
         <v/>
       </c>
       <c r="J23" s="7" t="n"/>
-      <c r="K23" s="7" t="n"/>
-      <c r="L23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n"/>
@@ -3815,8 +2453,6 @@
         <v/>
       </c>
       <c r="J24" s="7" t="n"/>
-      <c r="K24" s="7" t="n"/>
-      <c r="L24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -3832,8 +2468,6 @@
         <v/>
       </c>
       <c r="J25" s="7" t="n"/>
-      <c r="K25" s="7" t="n"/>
-      <c r="L25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n"/>
@@ -3849,8 +2483,6 @@
         <v/>
       </c>
       <c r="J26" s="7" t="n"/>
-      <c r="K26" s="7" t="n"/>
-      <c r="L26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n"/>
@@ -3866,8 +2498,6 @@
         <v/>
       </c>
       <c r="J27" s="7" t="n"/>
-      <c r="K27" s="7" t="n"/>
-      <c r="L27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n"/>
@@ -3883,8 +2513,6 @@
         <v/>
       </c>
       <c r="J28" s="7" t="n"/>
-      <c r="K28" s="7" t="n"/>
-      <c r="L28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n"/>
@@ -3900,8 +2528,6 @@
         <v/>
       </c>
       <c r="J29" s="7" t="n"/>
-      <c r="K29" s="7" t="n"/>
-      <c r="L29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n"/>
@@ -3917,8 +2543,6 @@
         <v/>
       </c>
       <c r="J30" s="7" t="n"/>
-      <c r="K30" s="7" t="n"/>
-      <c r="L30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n"/>
@@ -3934,8 +2558,6 @@
         <v/>
       </c>
       <c r="J31" s="7" t="n"/>
-      <c r="K31" s="7" t="n"/>
-      <c r="L31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n"/>
@@ -3951,8 +2573,6 @@
         <v/>
       </c>
       <c r="J32" s="7" t="n"/>
-      <c r="K32" s="7" t="n"/>
-      <c r="L32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n"/>
@@ -3968,8 +2588,6 @@
         <v/>
       </c>
       <c r="J33" s="7" t="n"/>
-      <c r="K33" s="7" t="n"/>
-      <c r="L33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n"/>
@@ -3985,8 +2603,6 @@
         <v/>
       </c>
       <c r="J34" s="7" t="n"/>
-      <c r="K34" s="7" t="n"/>
-      <c r="L34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n"/>
@@ -4002,8 +2618,6 @@
         <v/>
       </c>
       <c r="J35" s="7" t="n"/>
-      <c r="K35" s="7" t="n"/>
-      <c r="L35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n"/>
@@ -4019,8 +2633,6 @@
         <v/>
       </c>
       <c r="J36" s="7" t="n"/>
-      <c r="K36" s="7" t="n"/>
-      <c r="L36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -4036,8 +2648,6 @@
         <v/>
       </c>
       <c r="J37" s="7" t="n"/>
-      <c r="K37" s="7" t="n"/>
-      <c r="L37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n"/>
@@ -4053,8 +2663,6 @@
         <v/>
       </c>
       <c r="J38" s="7" t="n"/>
-      <c r="K38" s="7" t="n"/>
-      <c r="L38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n"/>
@@ -4070,8 +2678,6 @@
         <v/>
       </c>
       <c r="J39" s="7" t="n"/>
-      <c r="K39" s="7" t="n"/>
-      <c r="L39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n"/>
@@ -4087,8 +2693,6 @@
         <v/>
       </c>
       <c r="J40" s="7" t="n"/>
-      <c r="K40" s="7" t="n"/>
-      <c r="L40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n"/>
@@ -4104,8 +2708,6 @@
         <v/>
       </c>
       <c r="J41" s="7" t="n"/>
-      <c r="K41" s="7" t="n"/>
-      <c r="L41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n"/>
@@ -4121,8 +2723,6 @@
         <v/>
       </c>
       <c r="J42" s="7" t="n"/>
-      <c r="K42" s="7" t="n"/>
-      <c r="L42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n"/>
@@ -4138,8 +2738,6 @@
         <v/>
       </c>
       <c r="J43" s="7" t="n"/>
-      <c r="K43" s="7" t="n"/>
-      <c r="L43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n"/>
@@ -4155,8 +2753,6 @@
         <v/>
       </c>
       <c r="J44" s="7" t="n"/>
-      <c r="K44" s="7" t="n"/>
-      <c r="L44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n"/>
@@ -4172,8 +2768,6 @@
         <v/>
       </c>
       <c r="J45" s="7" t="n"/>
-      <c r="K45" s="7" t="n"/>
-      <c r="L45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n"/>
@@ -4189,8 +2783,6 @@
         <v/>
       </c>
       <c r="J46" s="7" t="n"/>
-      <c r="K46" s="7" t="n"/>
-      <c r="L46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n"/>
@@ -4206,8 +2798,6 @@
         <v/>
       </c>
       <c r="J47" s="7" t="n"/>
-      <c r="K47" s="7" t="n"/>
-      <c r="L47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n"/>
@@ -4223,8 +2813,6 @@
         <v/>
       </c>
       <c r="J48" s="7" t="n"/>
-      <c r="K48" s="7" t="n"/>
-      <c r="L48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="n"/>
@@ -4240,8 +2828,6 @@
         <v/>
       </c>
       <c r="J49" s="7" t="n"/>
-      <c r="K49" s="7" t="n"/>
-      <c r="L49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n"/>
@@ -4257,8 +2843,6 @@
         <v/>
       </c>
       <c r="J50" s="7" t="n"/>
-      <c r="K50" s="7" t="n"/>
-      <c r="L50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="n"/>
@@ -4274,8 +2858,6 @@
         <v/>
       </c>
       <c r="J51" s="7" t="n"/>
-      <c r="K51" s="7" t="n"/>
-      <c r="L51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n"/>
@@ -4291,8 +2873,6 @@
         <v/>
       </c>
       <c r="J52" s="7" t="n"/>
-      <c r="K52" s="7" t="n"/>
-      <c r="L52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="n"/>
@@ -4308,8 +2888,6 @@
         <v/>
       </c>
       <c r="J53" s="7" t="n"/>
-      <c r="K53" s="7" t="n"/>
-      <c r="L53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n"/>
@@ -4325,8 +2903,6 @@
         <v/>
       </c>
       <c r="J54" s="7" t="n"/>
-      <c r="K54" s="7" t="n"/>
-      <c r="L54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="n"/>
@@ -4342,8 +2918,6 @@
         <v/>
       </c>
       <c r="J55" s="7" t="n"/>
-      <c r="K55" s="7" t="n"/>
-      <c r="L55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n"/>
@@ -4359,8 +2933,6 @@
         <v/>
       </c>
       <c r="J56" s="7" t="n"/>
-      <c r="K56" s="7" t="n"/>
-      <c r="L56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="n"/>
@@ -4376,8 +2948,6 @@
         <v/>
       </c>
       <c r="J57" s="7" t="n"/>
-      <c r="K57" s="7" t="n"/>
-      <c r="L57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n"/>
@@ -4393,8 +2963,6 @@
         <v/>
       </c>
       <c r="J58" s="7" t="n"/>
-      <c r="K58" s="7" t="n"/>
-      <c r="L58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="n"/>
@@ -4410,8 +2978,6 @@
         <v/>
       </c>
       <c r="J59" s="7" t="n"/>
-      <c r="K59" s="7" t="n"/>
-      <c r="L59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n"/>
@@ -4427,8 +2993,6 @@
         <v/>
       </c>
       <c r="J60" s="7" t="n"/>
-      <c r="K60" s="7" t="n"/>
-      <c r="L60" s="7" t="n"/>
     </row>
     <row r="61">
       <c r="I61" s="10">
@@ -10077,12 +8641,21 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="E2:E3000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$B$1:$B$7</formula1>
+  <dataValidations count="5">
+    <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
+      <formula1>='Categories'!$A$3:$A$1000</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L3000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
-      <formula1>=Lists!$C$1:$C$2</formula1>
+    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
+      <formula1>='Collections'!$B$3:$B$1000</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
+      <formula1>=Lists!$A$1:$A$7</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
+      <formula1>='Warehouses'!$A$3:$A$1000</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Choose a value from the dropdown." type="list">
+      <formula1>=Lists!$B$1:$B$2</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10095,21 +8668,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>Plank</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
-        <is>
-          <t>Plank</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -10118,15 +8686,10 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AC4</t>
+          <t>Tile</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
-        <is>
-          <t>Tile</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
         <is>
           <t>Discontinued</t>
         </is>
@@ -10135,11 +8698,6 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AC5</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
           <t>Herringbone</t>
         </is>
       </c>
@@ -10147,31 +8705,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AC6</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
           <t>Chevron</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Board</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Profile</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Other</t>
         </is>

</xml_diff>

<commit_message>
EGO Master R4: the quantity rule (sq ft needed + wastage -> whole boxes -> sq ft supplied, rate per sq ft; accessories per piece or rft) across opportunity, order, PI, portal, Big E fulfilment, field app (build 1b88d5c779)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ego/EGO-Inventory-Upload-Template.xlsx
+++ b/ego/EGO-Inventory-Upload-Template.xlsx
@@ -554,7 +554,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>On Collections, fill the box size in square feet OR square metres. Square feet in stock is then worked out by itself, in this file and in EGO Master.</t>
+          <t>On Collections, fill the box size in sq ft OR square metres. Sq ft in stock is then worked out by itself, in this file and in EGO Master.</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>One row per collection (Divine, Delta, Slim Chevron...): its category, its box size in square feet or square metres, then the specifications all its designs share.</t>
+          <t>One row per collection (Divine, Delta, Slim Chevron...): its category, its box size in sq ft or square metres, then the specifications all its designs share.</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>One row per design per warehouse: category, collection, design, code, type, colour, the warehouse and the boxes there today. Square feet are worked out. After this, stock changes inside EGO Master with Stock in / out.</t>
+          <t>One row per design per warehouse: category, collection, design, code, type, colour, the warehouse and the boxes there today. Sq ft are worked out. After this, stock changes inside EGO Master with Stock in / out.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EGO Master R5: complaint photos + batch + installed by, telesales see every dealer, quotation uploads, Priority calls, role access per the 17 Oct ruling
</commit_message>
<xml_diff>
--- a/ego/EGO-Inventory-Upload-Template.xlsx
+++ b/ego/EGO-Inventory-Upload-Template.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>EGO-INV-3</t>
+          <t>EGO-INV-4</t>
         </is>
       </c>
     </row>
@@ -728,7 +728,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>Square feet in stock</t>
+          <t>Sq ft in stock</t>
         </is>
       </c>
       <c r="B24" s="4">
@@ -997,7 +997,7 @@
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="33" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -1018,12 +1018,12 @@
       </c>
       <c r="C1" s="8" t="inlineStr">
         <is>
-          <t>Box size in square feet</t>
+          <t>Box size in sq ft</t>
         </is>
       </c>
       <c r="D1" s="8" t="inlineStr">
         <is>
-          <t>Box size in square metres (fill this OR square feet)</t>
+          <t>Box size in square metres (fill this OR sq ft)</t>
         </is>
       </c>
       <c r="E1" s="8" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="I1" s="8" t="inlineStr">
         <is>
-          <t>Square feet in this warehouse (worked out, do not type)</t>
+          <t>Sq ft in this warehouse (worked out, do not type)</t>
         </is>
       </c>
       <c r="J1" s="8" t="inlineStr">

</xml_diff>